<commit_message>
fix: update README and add mock tables
</commit_message>
<xml_diff>
--- a/data/prices.xlsx
+++ b/data/prices.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,7 +448,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -456,14 +456,16 @@
           <t>PETR4</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>34.9664</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>35,30</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -472,13 +474,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>68.8086</v>
+        <v>69.0294</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -488,14 +490,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>29,64</t>
+          <t>29,72</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -505,374 +507,513 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>121,60</t>
+          <t>122.18</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>USD/BRL</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>5.0561</v>
+          <t>ABEV3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>14,83</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NTNB 2035</t>
+          <t>WEGE3</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.113,54</t>
+          <t>38.97</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PETR4</t>
+          <t>BBAS3</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>34.8047</v>
+        <v>52.442</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>VALE3</t>
+          <t>PETR4</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>68.1521</v>
+        <v>35.4455</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ITUB4</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>29.7023</v>
+          <t>VALE3</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>67,95</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BOVA11</t>
+          <t>ITUB4</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>122.6822</v>
+        <v>29.8694</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>USD/BRL</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>5.0925</v>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>123.88</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NTNB 2035</t>
+          <t>ABEV3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>5.085,40</t>
+          <t>15,11</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PETR4</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>35.0309</v>
+          <t>WEGE3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>38.14</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>VALE3</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>68.419</v>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>52,67</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ITUB4</t>
+          <t>PETR4</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>29.5582</v>
+        <v>35.3166</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>USD/BRL</t>
+          <t>VALE3</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>5,07</t>
+          <t>68.92</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>NTNB 2035</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>5076.203</v>
+          <t>ITUB4</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>29.84</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PETR4</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>35.3335</v>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>123,84</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>VALE3</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>67.86020000000001</v>
+          <t>ABEV3</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>15.16</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ITUB4</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>29.5555</v>
+          <t>WEGE3</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>38.75</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BOVA11</t>
+          <t>BBAS3</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>122.1152</v>
+        <v>51.5028</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>USD/BRL</t>
+          <t>PETR4</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5.0918</v>
+        <v>35.3945</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>NTNB 2035</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>5133.0539</v>
+          <t>VALE3</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>69,34</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PETR4</t>
+          <t>ITUB4</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>35.1268</v>
+        <v>30.1293</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>VALE3</t>
+          <t>BOVA11</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>68.426</v>
+        <v>122.7444</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ITUB4</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>29.4822</v>
+          <t>ABEV3</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>14,80</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BOVA11</t>
+          <t>WEGE3</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>121.6031</v>
+        <v>38.8391</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>NTNB 2035</t>
+          <t>BBAS3</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>5103.7429</v>
+        <v>52.0594</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>35,02</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>VALE3</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>68.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ITUB4</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>29.39</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>120.7296</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ABEV3</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>15,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>WEGE3</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>38,45</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>51.43</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>